<commit_message>
Stage 8 fixes: B-038
</commit_message>
<xml_diff>
--- a/output/archive/BrindlewytheData/Finance/Pricing/2026/screening_prices_2026_DRAFT_v3.xlsx
+++ b/output/archive/BrindlewytheData/Finance/Pricing/2026/screening_prices_2026_DRAFT_v3.xlsx
@@ -523,10 +523,8 @@
           <t>per compound</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>[TBC]</t>
-        </is>
+      <c r="D5" s="2" t="n">
+        <v>200</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -550,10 +548,8 @@
           <t>per compound</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>[TBC]</t>
-        </is>
+      <c r="D6" s="2" t="n">
+        <v>120</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -574,13 +570,11 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>per compound</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>[TBC]</t>
-        </is>
+          <t>per compound (panel)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1550</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -669,7 +663,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>[TBC]</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
@@ -687,7 +681,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>[TBC]</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -707,7 +701,11 @@
           <t>31 and above</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>5% &gt;30 cpds; 10% &gt;80 cpds</t>
+        </is>
+      </c>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6"/>

</xml_diff>